<commit_message>
Document single-asset volatility convention in methodology
Input vols are single-asset, not index-level (index = portfolio vol with
idiosyncratic risk diversified away plus appraisal smoothing). The model
prices one representative asset per sector — one deal, one loan — so
inputs sitting well above index vols is by design, and risk metrics
describe standalone assets. Validate inputs against property-level data.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TESTDCF8_test7.xlsx
+++ b/TESTDCF8_test7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f2d3817d0f7987d/Desktop/stochastic_model_sandbox/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{15C01B17-746E-4ABF-A7BF-674A9D12EB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8111480D-4B61-471E-AE4B-6293C3761C5F}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{15C01B17-746E-4ABF-A7BF-674A9D12EB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5DC267-9BE8-4C7F-8450-E11C60C18ED0}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="23020" windowHeight="14620" xr2:uid="{1F92A932-4862-4E03-8261-7584EC3D15AE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{1F92A932-4862-4E03-8261-7584EC3D15AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -521,6 +521,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1535,7 +1539,7 @@
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="K10" s="8">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="L10" s="11">
         <v>0.10525647584898666</v>
@@ -1679,7 +1683,7 @@
         <v>0.11849999999999999</v>
       </c>
       <c r="K12" s="8">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="L12" s="11">
         <v>9.5687705317260591E-2</v>

</xml_diff>